<commit_message>
apply new ascii_to_csv into 3 location
</commit_message>
<xml_diff>
--- a/Dataset/Data Buoys/4N90E/EXCEL/w4n90e_dy.xlsx
+++ b/Dataset/Data Buoys/4N90E/EXCEL/w4n90e_dy.xlsx
@@ -451,6 +451,12 @@
       <c r="D2">
         <v>16</v>
       </c>
+      <c r="E2">
+        <v>-2.4</v>
+      </c>
+      <c r="F2">
+        <v>-2.8</v>
+      </c>
       <c r="G2">
         <v>3.6</v>
       </c>
@@ -471,6 +477,12 @@
       <c r="D3">
         <v>17</v>
       </c>
+      <c r="E3">
+        <v>-1.3</v>
+      </c>
+      <c r="F3">
+        <v>-0.8</v>
+      </c>
       <c r="G3">
         <v>1.5</v>
       </c>
@@ -517,6 +529,9 @@
       <c r="D5">
         <v>19</v>
       </c>
+      <c r="E5">
+        <v>-0.9</v>
+      </c>
       <c r="F5">
         <v>2.8</v>
       </c>
@@ -569,6 +584,9 @@
       <c r="E7">
         <v>4.2</v>
       </c>
+      <c r="F7">
+        <v>-1.9</v>
+      </c>
       <c r="G7">
         <v>4.7</v>
       </c>
@@ -592,6 +610,9 @@
       <c r="E8">
         <v>3.4</v>
       </c>
+      <c r="F8">
+        <v>-1.9</v>
+      </c>
       <c r="G8">
         <v>3.9</v>
       </c>
@@ -612,6 +633,9 @@
       <c r="D9">
         <v>23</v>
       </c>
+      <c r="E9">
+        <v>-1.5</v>
+      </c>
       <c r="F9">
         <v>2.1</v>
       </c>
@@ -635,6 +659,9 @@
       <c r="D10">
         <v>24</v>
       </c>
+      <c r="E10">
+        <v>-0.6</v>
+      </c>
       <c r="F10">
         <v>1.9</v>
       </c>
@@ -687,6 +714,9 @@
       <c r="E12">
         <v>0.6</v>
       </c>
+      <c r="F12">
+        <v>-1.3</v>
+      </c>
       <c r="G12">
         <v>1.4</v>
       </c>
@@ -707,6 +737,9 @@
       <c r="D13">
         <v>8</v>
       </c>
+      <c r="E13">
+        <v>-0.3</v>
+      </c>
       <c r="F13">
         <v>2.1</v>
       </c>
@@ -782,6 +815,9 @@
       <c r="D16">
         <v>11</v>
       </c>
+      <c r="E16">
+        <v>-0.7</v>
+      </c>
       <c r="F16">
         <v>0.9</v>
       </c>
@@ -808,6 +844,9 @@
       <c r="E17">
         <v>1.5</v>
       </c>
+      <c r="F17">
+        <v>-0.6</v>
+      </c>
       <c r="G17">
         <v>1.6</v>
       </c>
@@ -883,6 +922,9 @@
       <c r="E20">
         <v>2.9</v>
       </c>
+      <c r="F20">
+        <v>-0.7</v>
+      </c>
       <c r="G20">
         <v>3</v>
       </c>
@@ -958,6 +1000,9 @@
       <c r="E23">
         <v>2.5</v>
       </c>
+      <c r="F23">
+        <v>-3.1</v>
+      </c>
       <c r="G23">
         <v>4</v>
       </c>
@@ -981,6 +1026,9 @@
       <c r="E24">
         <v>4.6</v>
       </c>
+      <c r="F24">
+        <v>-6</v>
+      </c>
       <c r="G24">
         <v>7.5</v>
       </c>
@@ -1004,6 +1052,9 @@
       <c r="E25">
         <v>8.1</v>
       </c>
+      <c r="F25">
+        <v>-0.7</v>
+      </c>
       <c r="G25">
         <v>8.199999999999999</v>
       </c>
@@ -1027,6 +1078,9 @@
       <c r="E26">
         <v>7.8</v>
       </c>
+      <c r="F26">
+        <v>-3.3</v>
+      </c>
       <c r="G26">
         <v>8.5</v>
       </c>
@@ -1050,6 +1104,9 @@
       <c r="E27">
         <v>8.1</v>
       </c>
+      <c r="F27">
+        <v>-0.3</v>
+      </c>
       <c r="G27">
         <v>8.1</v>
       </c>
@@ -1281,6 +1338,9 @@
       <c r="E36">
         <v>3.1</v>
       </c>
+      <c r="F36">
+        <v>-0.7</v>
+      </c>
       <c r="G36">
         <v>3.2</v>
       </c>
@@ -1408,6 +1468,9 @@
       <c r="E41">
         <v>3.5</v>
       </c>
+      <c r="F41">
+        <v>-1.1</v>
+      </c>
       <c r="G41">
         <v>3.7</v>
       </c>
@@ -1457,6 +1520,9 @@
       <c r="E43">
         <v>8.1</v>
       </c>
+      <c r="F43">
+        <v>-0.5</v>
+      </c>
       <c r="G43">
         <v>8.199999999999999</v>
       </c>
@@ -1662,6 +1728,9 @@
       <c r="E51">
         <v>0</v>
       </c>
+      <c r="F51">
+        <v>-0.6</v>
+      </c>
       <c r="G51">
         <v>0.6</v>
       </c>
@@ -1682,6 +1751,12 @@
       <c r="D52">
         <v>16</v>
       </c>
+      <c r="E52">
+        <v>-1.9</v>
+      </c>
+      <c r="F52">
+        <v>-2.7</v>
+      </c>
       <c r="G52">
         <v>3.4</v>
       </c>
@@ -1702,6 +1777,12 @@
       <c r="D53">
         <v>17</v>
       </c>
+      <c r="E53">
+        <v>-2.2</v>
+      </c>
+      <c r="F53">
+        <v>-1.9</v>
+      </c>
       <c r="G53">
         <v>2.9</v>
       </c>
@@ -1722,6 +1803,9 @@
       <c r="D54">
         <v>18</v>
       </c>
+      <c r="E54">
+        <v>-1.5</v>
+      </c>
       <c r="F54">
         <v>1</v>
       </c>
@@ -1745,6 +1829,9 @@
       <c r="D55">
         <v>19</v>
       </c>
+      <c r="E55">
+        <v>-1.5</v>
+      </c>
       <c r="F55">
         <v>2.6</v>
       </c>
@@ -1768,6 +1855,9 @@
       <c r="D56">
         <v>20</v>
       </c>
+      <c r="E56">
+        <v>-1.7</v>
+      </c>
       <c r="F56">
         <v>2</v>
       </c>
@@ -1791,6 +1881,9 @@
       <c r="D57">
         <v>21</v>
       </c>
+      <c r="E57">
+        <v>-2.5</v>
+      </c>
       <c r="F57">
         <v>3.4</v>
       </c>
@@ -1814,6 +1907,9 @@
       <c r="D58">
         <v>22</v>
       </c>
+      <c r="E58">
+        <v>-0.9</v>
+      </c>
       <c r="F58">
         <v>1.5</v>
       </c>
@@ -1840,6 +1936,9 @@
       <c r="E59">
         <v>2.5</v>
       </c>
+      <c r="F59">
+        <v>-0.9</v>
+      </c>
       <c r="G59">
         <v>2.7</v>
       </c>
@@ -1863,6 +1962,9 @@
       <c r="E60">
         <v>2.1</v>
       </c>
+      <c r="F60">
+        <v>-0.1</v>
+      </c>
       <c r="G60">
         <v>2.1</v>
       </c>
@@ -1961,6 +2063,12 @@
       <c r="D64">
         <v>28</v>
       </c>
+      <c r="E64">
+        <v>-0.1</v>
+      </c>
+      <c r="F64">
+        <v>-2.9</v>
+      </c>
       <c r="G64">
         <v>2.9</v>
       </c>
@@ -1981,6 +2089,12 @@
       <c r="D65">
         <v>29</v>
       </c>
+      <c r="E65">
+        <v>-1.4</v>
+      </c>
+      <c r="F65">
+        <v>-1.5</v>
+      </c>
       <c r="G65">
         <v>2.1</v>
       </c>
@@ -2001,6 +2115,9 @@
       <c r="D66">
         <v>30</v>
       </c>
+      <c r="E66">
+        <v>-2.5</v>
+      </c>
       <c r="F66">
         <v>0.3</v>
       </c>
@@ -2024,6 +2141,12 @@
       <c r="D67">
         <v>1</v>
       </c>
+      <c r="E67">
+        <v>-0.1</v>
+      </c>
+      <c r="F67">
+        <v>-3.3</v>
+      </c>
       <c r="G67">
         <v>3.3</v>
       </c>
@@ -2044,6 +2167,12 @@
       <c r="D68">
         <v>2</v>
       </c>
+      <c r="E68">
+        <v>-2.9</v>
+      </c>
+      <c r="F68">
+        <v>-6.8</v>
+      </c>
       <c r="G68">
         <v>7.5</v>
       </c>
@@ -2064,6 +2193,12 @@
       <c r="D69">
         <v>3</v>
       </c>
+      <c r="E69">
+        <v>-8.1</v>
+      </c>
+      <c r="F69">
+        <v>-6.4</v>
+      </c>
       <c r="G69">
         <v>10.3</v>
       </c>
@@ -2084,6 +2219,12 @@
       <c r="D70">
         <v>4</v>
       </c>
+      <c r="E70">
+        <v>-8.1</v>
+      </c>
+      <c r="F70">
+        <v>-5.2</v>
+      </c>
       <c r="G70">
         <v>9.6</v>
       </c>
@@ -2104,6 +2245,12 @@
       <c r="D71">
         <v>5</v>
       </c>
+      <c r="E71">
+        <v>-7.4</v>
+      </c>
+      <c r="F71">
+        <v>-3.8</v>
+      </c>
       <c r="G71">
         <v>8.300000000000001</v>
       </c>
@@ -2124,6 +2271,12 @@
       <c r="D72">
         <v>6</v>
       </c>
+      <c r="E72">
+        <v>-6.6</v>
+      </c>
+      <c r="F72">
+        <v>-4.6</v>
+      </c>
       <c r="G72">
         <v>8</v>
       </c>
@@ -2144,6 +2297,12 @@
       <c r="D73">
         <v>7</v>
       </c>
+      <c r="E73">
+        <v>-6.2</v>
+      </c>
+      <c r="F73">
+        <v>-3.6</v>
+      </c>
       <c r="G73">
         <v>7.2</v>
       </c>
@@ -2190,6 +2349,12 @@
       <c r="D75">
         <v>9</v>
       </c>
+      <c r="E75">
+        <v>-3.8</v>
+      </c>
+      <c r="F75">
+        <v>-0.9</v>
+      </c>
       <c r="G75">
         <v>3.9</v>
       </c>
@@ -2210,6 +2375,9 @@
       <c r="D76">
         <v>10</v>
       </c>
+      <c r="E76">
+        <v>-2.1</v>
+      </c>
       <c r="F76">
         <v>2</v>
       </c>
@@ -2233,6 +2401,9 @@
       <c r="D77">
         <v>11</v>
       </c>
+      <c r="E77">
+        <v>-4.7</v>
+      </c>
       <c r="F77">
         <v>2.2</v>
       </c>
@@ -2256,6 +2427,9 @@
       <c r="D78">
         <v>12</v>
       </c>
+      <c r="E78">
+        <v>-1.9</v>
+      </c>
       <c r="F78">
         <v>2.8</v>
       </c>
@@ -2282,6 +2456,9 @@
       <c r="E79">
         <v>1.1</v>
       </c>
+      <c r="F79">
+        <v>-2</v>
+      </c>
       <c r="G79">
         <v>2.3</v>
       </c>
@@ -2305,6 +2482,9 @@
       <c r="E80">
         <v>3.3</v>
       </c>
+      <c r="F80">
+        <v>-0.9</v>
+      </c>
       <c r="G80">
         <v>3.4</v>
       </c>
@@ -2325,6 +2505,12 @@
       <c r="D81">
         <v>15</v>
       </c>
+      <c r="E81">
+        <v>-1.5</v>
+      </c>
+      <c r="F81">
+        <v>-3.5</v>
+      </c>
       <c r="G81">
         <v>3.8</v>
       </c>
@@ -2345,6 +2531,9 @@
       <c r="D82">
         <v>16</v>
       </c>
+      <c r="E82">
+        <v>-1.9</v>
+      </c>
       <c r="F82">
         <v>2</v>
       </c>
@@ -2368,6 +2557,9 @@
       <c r="D83">
         <v>17</v>
       </c>
+      <c r="E83">
+        <v>-3.9</v>
+      </c>
       <c r="F83">
         <v>1.7</v>
       </c>
@@ -2391,6 +2583,12 @@
       <c r="D84">
         <v>18</v>
       </c>
+      <c r="E84">
+        <v>-4.2</v>
+      </c>
+      <c r="F84">
+        <v>-0.6</v>
+      </c>
       <c r="G84">
         <v>4.3</v>
       </c>
@@ -2411,6 +2609,12 @@
       <c r="D85">
         <v>19</v>
       </c>
+      <c r="E85">
+        <v>-2.5</v>
+      </c>
+      <c r="F85">
+        <v>-3.3</v>
+      </c>
       <c r="G85">
         <v>4.2</v>
       </c>
@@ -2431,6 +2635,12 @@
       <c r="D86">
         <v>20</v>
       </c>
+      <c r="E86">
+        <v>-4</v>
+      </c>
+      <c r="F86">
+        <v>-0.8</v>
+      </c>
       <c r="G86">
         <v>4.1</v>
       </c>
@@ -2451,6 +2661,12 @@
       <c r="D87">
         <v>21</v>
       </c>
+      <c r="E87">
+        <v>-2.4</v>
+      </c>
+      <c r="F87">
+        <v>-1.1</v>
+      </c>
       <c r="G87">
         <v>2.7</v>
       </c>
@@ -2471,6 +2687,12 @@
       <c r="D88">
         <v>22</v>
       </c>
+      <c r="E88">
+        <v>-1.7</v>
+      </c>
+      <c r="F88">
+        <v>-0.5</v>
+      </c>
       <c r="G88">
         <v>1.8</v>
       </c>
@@ -2520,6 +2742,9 @@
       <c r="E90">
         <v>4.7</v>
       </c>
+      <c r="F90">
+        <v>-2.6</v>
+      </c>
       <c r="G90">
         <v>5.4</v>
       </c>
@@ -2540,6 +2765,12 @@
       <c r="D91">
         <v>25</v>
       </c>
+      <c r="E91">
+        <v>-1.3</v>
+      </c>
+      <c r="F91">
+        <v>-3.5</v>
+      </c>
       <c r="G91">
         <v>3.7</v>
       </c>
@@ -2560,6 +2791,12 @@
       <c r="D92">
         <v>26</v>
       </c>
+      <c r="E92">
+        <v>-0.6</v>
+      </c>
+      <c r="F92">
+        <v>-4.8</v>
+      </c>
       <c r="G92">
         <v>4.9</v>
       </c>
@@ -2583,6 +2820,9 @@
       <c r="E93">
         <v>1.8</v>
       </c>
+      <c r="F93">
+        <v>-5.5</v>
+      </c>
       <c r="G93">
         <v>5.8</v>
       </c>
@@ -2606,6 +2846,9 @@
       <c r="E94">
         <v>3.4</v>
       </c>
+      <c r="F94">
+        <v>-5.5</v>
+      </c>
       <c r="G94">
         <v>6.4</v>
       </c>
@@ -2629,6 +2872,9 @@
       <c r="E95">
         <v>0.4</v>
       </c>
+      <c r="F95">
+        <v>-4.8</v>
+      </c>
       <c r="G95">
         <v>4.8</v>
       </c>
@@ -2649,6 +2895,12 @@
       <c r="D96">
         <v>30</v>
       </c>
+      <c r="E96">
+        <v>-0.1</v>
+      </c>
+      <c r="F96">
+        <v>-4</v>
+      </c>
       <c r="G96">
         <v>4</v>
       </c>
@@ -2669,6 +2921,12 @@
       <c r="D97">
         <v>31</v>
       </c>
+      <c r="E97">
+        <v>-0.3</v>
+      </c>
+      <c r="F97">
+        <v>-2.9</v>
+      </c>
       <c r="G97">
         <v>2.9</v>
       </c>
@@ -2689,6 +2947,12 @@
       <c r="D98">
         <v>1</v>
       </c>
+      <c r="E98">
+        <v>-1.7</v>
+      </c>
+      <c r="F98">
+        <v>-0.5</v>
+      </c>
       <c r="G98">
         <v>1.8</v>
       </c>
@@ -2709,6 +2973,9 @@
       <c r="D99">
         <v>2</v>
       </c>
+      <c r="E99">
+        <v>-0.9</v>
+      </c>
       <c r="F99">
         <v>1.5</v>
       </c>
@@ -2732,6 +2999,9 @@
       <c r="D100">
         <v>3</v>
       </c>
+      <c r="E100">
+        <v>-2.1</v>
+      </c>
       <c r="F100">
         <v>2.2</v>
       </c>
@@ -2781,6 +3051,12 @@
       <c r="D102">
         <v>5</v>
       </c>
+      <c r="E102">
+        <v>-0.9</v>
+      </c>
+      <c r="F102">
+        <v>-0.3</v>
+      </c>
       <c r="G102">
         <v>1</v>
       </c>
@@ -2801,6 +3077,9 @@
       <c r="D103">
         <v>5</v>
       </c>
+      <c r="E103">
+        <v>-0.5</v>
+      </c>
       <c r="F103">
         <v>3</v>
       </c>
@@ -2850,6 +3129,9 @@
       <c r="D105">
         <v>7</v>
       </c>
+      <c r="E105">
+        <v>-1.6</v>
+      </c>
       <c r="F105">
         <v>5</v>
       </c>
@@ -2873,6 +3155,9 @@
       <c r="D106">
         <v>8</v>
       </c>
+      <c r="E106">
+        <v>-2</v>
+      </c>
       <c r="F106">
         <v>5.9</v>
       </c>
@@ -2977,6 +3262,9 @@
       <c r="E110">
         <v>1.7</v>
       </c>
+      <c r="F110">
+        <v>-1</v>
+      </c>
       <c r="G110">
         <v>2</v>
       </c>
@@ -3000,6 +3288,9 @@
       <c r="E111">
         <v>4.5</v>
       </c>
+      <c r="F111">
+        <v>-1.4</v>
+      </c>
       <c r="G111">
         <v>4.7</v>
       </c>
@@ -4895,6 +5186,9 @@
       <c r="E184">
         <v>5.6</v>
       </c>
+      <c r="F184">
+        <v>-0.4</v>
+      </c>
       <c r="G184">
         <v>5.6</v>
       </c>
@@ -4918,6 +5212,9 @@
       <c r="E185">
         <v>5.8</v>
       </c>
+      <c r="F185">
+        <v>-1.2</v>
+      </c>
       <c r="G185">
         <v>5.9</v>
       </c>
@@ -4941,6 +5238,9 @@
       <c r="E186">
         <v>3.6</v>
       </c>
+      <c r="F186">
+        <v>-0.1</v>
+      </c>
       <c r="G186">
         <v>3.6</v>
       </c>
@@ -4964,6 +5264,9 @@
       <c r="E187">
         <v>3.9</v>
       </c>
+      <c r="F187">
+        <v>-0.7</v>
+      </c>
       <c r="G187">
         <v>3.9</v>
       </c>
@@ -5013,6 +5316,9 @@
       <c r="E189">
         <v>5.6</v>
       </c>
+      <c r="F189">
+        <v>-1.2</v>
+      </c>
       <c r="G189">
         <v>5.8</v>
       </c>
@@ -5660,6 +5966,9 @@
       <c r="E214">
         <v>6.2</v>
       </c>
+      <c r="F214">
+        <v>-0.8</v>
+      </c>
       <c r="G214">
         <v>6.2</v>
       </c>
@@ -5735,6 +6044,9 @@
       <c r="E217">
         <v>4.5</v>
       </c>
+      <c r="F217">
+        <v>-1.4</v>
+      </c>
       <c r="G217">
         <v>4.7</v>
       </c>
@@ -5888,6 +6200,9 @@
       <c r="E223">
         <v>8</v>
       </c>
+      <c r="F223">
+        <v>-2.3</v>
+      </c>
       <c r="G223">
         <v>8.300000000000001</v>
       </c>
@@ -5911,6 +6226,9 @@
       <c r="E224">
         <v>6.7</v>
       </c>
+      <c r="F224">
+        <v>-4.1</v>
+      </c>
       <c r="G224">
         <v>7.8</v>
       </c>
@@ -6064,6 +6382,9 @@
       <c r="E230">
         <v>2.9</v>
       </c>
+      <c r="F230">
+        <v>-1.3</v>
+      </c>
       <c r="G230">
         <v>3.2</v>
       </c>
@@ -6113,6 +6434,9 @@
       <c r="E232">
         <v>9</v>
       </c>
+      <c r="F232">
+        <v>-2.1</v>
+      </c>
       <c r="G232">
         <v>9.199999999999999</v>
       </c>
@@ -6136,6 +6460,9 @@
       <c r="E233">
         <v>4.6</v>
       </c>
+      <c r="F233">
+        <v>-0.4</v>
+      </c>
       <c r="G233">
         <v>4.7</v>
       </c>
@@ -6159,6 +6486,9 @@
       <c r="E234">
         <v>2.7</v>
       </c>
+      <c r="F234">
+        <v>-0.1</v>
+      </c>
       <c r="G234">
         <v>2.7</v>
       </c>
@@ -6234,6 +6564,9 @@
       <c r="E237">
         <v>1.5</v>
       </c>
+      <c r="F237">
+        <v>-0.4</v>
+      </c>
       <c r="G237">
         <v>1.6</v>
       </c>
@@ -6254,6 +6587,12 @@
       <c r="D238">
         <v>17</v>
       </c>
+      <c r="E238">
+        <v>-0.3</v>
+      </c>
+      <c r="F238">
+        <v>-2.1</v>
+      </c>
       <c r="G238">
         <v>2.1</v>
       </c>
@@ -6277,6 +6616,9 @@
       <c r="E239">
         <v>1.3</v>
       </c>
+      <c r="F239">
+        <v>-0.8</v>
+      </c>
       <c r="G239">
         <v>1.6</v>
       </c>
@@ -6300,6 +6642,9 @@
       <c r="E240">
         <v>0.3</v>
       </c>
+      <c r="F240">
+        <v>-0.7</v>
+      </c>
       <c r="G240">
         <v>0.8</v>
       </c>
@@ -6349,6 +6694,9 @@
       <c r="E242">
         <v>2.1</v>
       </c>
+      <c r="F242">
+        <v>-0.8</v>
+      </c>
       <c r="G242">
         <v>2.2</v>
       </c>
@@ -6398,6 +6746,9 @@
       <c r="E244">
         <v>6.2</v>
       </c>
+      <c r="F244">
+        <v>-0.6</v>
+      </c>
       <c r="G244">
         <v>6.2</v>
       </c>
@@ -6473,6 +6824,9 @@
       <c r="E247">
         <v>6.2</v>
       </c>
+      <c r="F247">
+        <v>-1</v>
+      </c>
       <c r="G247">
         <v>6.3</v>
       </c>
@@ -6496,6 +6850,9 @@
       <c r="E248">
         <v>8</v>
       </c>
+      <c r="F248">
+        <v>-2.3</v>
+      </c>
       <c r="G248">
         <v>8.300000000000001</v>
       </c>
@@ -6519,6 +6876,9 @@
       <c r="E249">
         <v>0.3</v>
       </c>
+      <c r="F249">
+        <v>-0.7</v>
+      </c>
       <c r="G249">
         <v>0.8</v>
       </c>
@@ -6539,6 +6899,12 @@
       <c r="D250">
         <v>29</v>
       </c>
+      <c r="E250">
+        <v>-2.6</v>
+      </c>
+      <c r="F250">
+        <v>-2.1</v>
+      </c>
       <c r="G250">
         <v>3.3</v>
       </c>
@@ -6559,6 +6925,9 @@
       <c r="D251">
         <v>30</v>
       </c>
+      <c r="E251">
+        <v>-3.7</v>
+      </c>
       <c r="F251">
         <v>0.9</v>
       </c>
@@ -6585,6 +6954,9 @@
       <c r="E252">
         <v>1.7</v>
       </c>
+      <c r="F252">
+        <v>-2.2</v>
+      </c>
       <c r="G252">
         <v>2.8</v>
       </c>
@@ -6608,6 +6980,9 @@
       <c r="E253">
         <v>3.9</v>
       </c>
+      <c r="F253">
+        <v>-3.7</v>
+      </c>
       <c r="G253">
         <v>5.4</v>
       </c>
@@ -6761,6 +7136,9 @@
       <c r="E259">
         <v>1.1</v>
       </c>
+      <c r="F259">
+        <v>-1</v>
+      </c>
       <c r="G259">
         <v>1.5</v>
       </c>
@@ -6836,6 +7214,9 @@
       <c r="E262">
         <v>4.8</v>
       </c>
+      <c r="F262">
+        <v>-0.2</v>
+      </c>
       <c r="G262">
         <v>4.8</v>
       </c>
@@ -6885,6 +7266,9 @@
       <c r="E264">
         <v>2.5</v>
       </c>
+      <c r="F264">
+        <v>-1.6</v>
+      </c>
       <c r="G264">
         <v>3</v>
       </c>
@@ -6905,6 +7289,12 @@
       <c r="D265">
         <v>14</v>
       </c>
+      <c r="E265">
+        <v>-0.3</v>
+      </c>
+      <c r="F265">
+        <v>-2.7</v>
+      </c>
       <c r="G265">
         <v>2.7</v>
       </c>
@@ -6928,6 +7318,9 @@
       <c r="E266">
         <v>0.1</v>
       </c>
+      <c r="F266">
+        <v>-3.2</v>
+      </c>
       <c r="G266">
         <v>3.3</v>
       </c>
@@ -6951,6 +7344,9 @@
       <c r="E267">
         <v>0.1</v>
       </c>
+      <c r="F267">
+        <v>-2.5</v>
+      </c>
       <c r="G267">
         <v>2.5</v>
       </c>
@@ -6971,6 +7367,12 @@
       <c r="D268">
         <v>17</v>
       </c>
+      <c r="E268">
+        <v>-0.6</v>
+      </c>
+      <c r="F268">
+        <v>-2.1</v>
+      </c>
       <c r="G268">
         <v>2.2</v>
       </c>
@@ -6991,6 +7393,12 @@
       <c r="D269">
         <v>18</v>
       </c>
+      <c r="E269">
+        <v>-1.8</v>
+      </c>
+      <c r="F269">
+        <v>-1.1</v>
+      </c>
       <c r="G269">
         <v>2.1</v>
       </c>
@@ -7011,6 +7419,12 @@
       <c r="D270">
         <v>19</v>
       </c>
+      <c r="E270">
+        <v>-0.8</v>
+      </c>
+      <c r="F270">
+        <v>-0.9</v>
+      </c>
       <c r="G270">
         <v>1.2</v>
       </c>
@@ -7031,6 +7445,9 @@
       <c r="D271">
         <v>20</v>
       </c>
+      <c r="E271">
+        <v>-1.7</v>
+      </c>
       <c r="F271">
         <v>0.8</v>
       </c>
@@ -7054,6 +7471,12 @@
       <c r="D272">
         <v>21</v>
       </c>
+      <c r="E272">
+        <v>-1.4</v>
+      </c>
+      <c r="F272">
+        <v>-2.5</v>
+      </c>
       <c r="G272">
         <v>2.9</v>
       </c>
@@ -7074,6 +7497,12 @@
       <c r="D273">
         <v>22</v>
       </c>
+      <c r="E273">
+        <v>-1.5</v>
+      </c>
+      <c r="F273">
+        <v>-0.3</v>
+      </c>
       <c r="G273">
         <v>1.5</v>
       </c>
@@ -7094,6 +7523,9 @@
       <c r="D274">
         <v>23</v>
       </c>
+      <c r="E274">
+        <v>-1.3</v>
+      </c>
       <c r="F274">
         <v>2.2</v>
       </c>
@@ -7143,6 +7575,9 @@
       <c r="D276">
         <v>25</v>
       </c>
+      <c r="E276">
+        <v>-0.5</v>
+      </c>
       <c r="F276">
         <v>1.1</v>
       </c>
@@ -7192,6 +7627,9 @@
       <c r="D278">
         <v>27</v>
       </c>
+      <c r="E278">
+        <v>-1.9</v>
+      </c>
       <c r="F278">
         <v>1.2</v>
       </c>
@@ -7215,6 +7653,9 @@
       <c r="D279">
         <v>28</v>
       </c>
+      <c r="E279">
+        <v>-1.7</v>
+      </c>
       <c r="F279">
         <v>2</v>
       </c>
@@ -7238,6 +7679,9 @@
       <c r="D280">
         <v>29</v>
       </c>
+      <c r="E280">
+        <v>-2.3</v>
+      </c>
       <c r="F280">
         <v>1.2</v>
       </c>
@@ -7264,6 +7708,9 @@
       <c r="E281">
         <v>0.5</v>
       </c>
+      <c r="F281">
+        <v>-1.1</v>
+      </c>
       <c r="G281">
         <v>1.2</v>
       </c>
@@ -7287,6 +7734,9 @@
       <c r="E282">
         <v>0.5</v>
       </c>
+      <c r="F282">
+        <v>-3.4</v>
+      </c>
       <c r="G282">
         <v>3.5</v>
       </c>
@@ -7310,6 +7760,9 @@
       <c r="E283">
         <v>0.1</v>
       </c>
+      <c r="F283">
+        <v>-1.7</v>
+      </c>
       <c r="G283">
         <v>1.7</v>
       </c>
@@ -7330,6 +7783,9 @@
       <c r="D284">
         <v>2</v>
       </c>
+      <c r="E284">
+        <v>-1.7</v>
+      </c>
       <c r="F284">
         <v>2</v>
       </c>
@@ -7353,6 +7809,9 @@
       <c r="D285">
         <v>3</v>
       </c>
+      <c r="E285">
+        <v>-2.5</v>
+      </c>
       <c r="F285">
         <v>1.4</v>
       </c>
@@ -7376,6 +7835,9 @@
       <c r="D286">
         <v>4</v>
       </c>
+      <c r="E286">
+        <v>-1.1</v>
+      </c>
       <c r="F286">
         <v>3.6</v>
       </c>
@@ -7399,6 +7861,9 @@
       <c r="D287">
         <v>5</v>
       </c>
+      <c r="E287">
+        <v>-0.9</v>
+      </c>
       <c r="F287">
         <v>3.8</v>
       </c>
@@ -7581,6 +8046,9 @@
       <c r="E294">
         <v>4.5</v>
       </c>
+      <c r="F294">
+        <v>-1.2</v>
+      </c>
       <c r="G294">
         <v>4.6</v>
       </c>
@@ -7604,6 +8072,9 @@
       <c r="E295">
         <v>0.5</v>
       </c>
+      <c r="F295">
+        <v>-2.7</v>
+      </c>
       <c r="G295">
         <v>2.7</v>
       </c>
@@ -7624,6 +8095,12 @@
       <c r="D296">
         <v>14</v>
       </c>
+      <c r="E296">
+        <v>-0.9</v>
+      </c>
+      <c r="F296">
+        <v>-0.3</v>
+      </c>
       <c r="G296">
         <v>0.9</v>
       </c>
@@ -7644,6 +8121,12 @@
       <c r="D297">
         <v>15</v>
       </c>
+      <c r="E297">
+        <v>-0.5</v>
+      </c>
+      <c r="F297">
+        <v>-0.3</v>
+      </c>
       <c r="G297">
         <v>0.6</v>
       </c>
@@ -7690,6 +8173,12 @@
       <c r="D299">
         <v>17</v>
       </c>
+      <c r="E299">
+        <v>-0.2</v>
+      </c>
+      <c r="F299">
+        <v>-1.3</v>
+      </c>
       <c r="G299">
         <v>1.3</v>
       </c>
@@ -7710,6 +8199,12 @@
       <c r="D300">
         <v>18</v>
       </c>
+      <c r="E300">
+        <v>-1.9</v>
+      </c>
+      <c r="F300">
+        <v>-2.9</v>
+      </c>
       <c r="G300">
         <v>3.5</v>
       </c>
@@ -7730,6 +8225,12 @@
       <c r="D301">
         <v>19</v>
       </c>
+      <c r="E301">
+        <v>-3.4</v>
+      </c>
+      <c r="F301">
+        <v>-4.3</v>
+      </c>
       <c r="G301">
         <v>5.5</v>
       </c>
@@ -7750,6 +8251,12 @@
       <c r="D302">
         <v>20</v>
       </c>
+      <c r="E302">
+        <v>-0.8</v>
+      </c>
+      <c r="F302">
+        <v>-4.8</v>
+      </c>
       <c r="G302">
         <v>4.9</v>
       </c>
@@ -7770,6 +8277,12 @@
       <c r="D303">
         <v>21</v>
       </c>
+      <c r="E303">
+        <v>-3.3</v>
+      </c>
+      <c r="F303">
+        <v>-3.5</v>
+      </c>
       <c r="G303">
         <v>4.8</v>
       </c>
@@ -7790,6 +8303,12 @@
       <c r="D304">
         <v>22</v>
       </c>
+      <c r="E304">
+        <v>-4.4</v>
+      </c>
+      <c r="F304">
+        <v>-5.7</v>
+      </c>
       <c r="G304">
         <v>7.2</v>
       </c>
@@ -7810,6 +8329,12 @@
       <c r="D305">
         <v>23</v>
       </c>
+      <c r="E305">
+        <v>-4.2</v>
+      </c>
+      <c r="F305">
+        <v>-4.1</v>
+      </c>
       <c r="G305">
         <v>5.9</v>
       </c>
@@ -7830,6 +8355,12 @@
       <c r="D306">
         <v>24</v>
       </c>
+      <c r="E306">
+        <v>-5.1</v>
+      </c>
+      <c r="F306">
+        <v>-2.6</v>
+      </c>
       <c r="G306">
         <v>5.7</v>
       </c>
@@ -7850,6 +8381,12 @@
       <c r="D307">
         <v>25</v>
       </c>
+      <c r="E307">
+        <v>-4.2</v>
+      </c>
+      <c r="F307">
+        <v>-1.1</v>
+      </c>
       <c r="G307">
         <v>4.3</v>
       </c>
@@ -7870,6 +8407,12 @@
       <c r="D308">
         <v>26</v>
       </c>
+      <c r="E308">
+        <v>-3.8</v>
+      </c>
+      <c r="F308">
+        <v>-0.7</v>
+      </c>
       <c r="G308">
         <v>3.9</v>
       </c>
@@ -7890,6 +8433,9 @@
       <c r="D309">
         <v>27</v>
       </c>
+      <c r="E309">
+        <v>-0.5</v>
+      </c>
       <c r="F309">
         <v>1.3</v>
       </c>
@@ -8719,6 +9265,9 @@
       <c r="D341">
         <v>7</v>
       </c>
+      <c r="E341">
+        <v>-0.6</v>
+      </c>
       <c r="F341">
         <v>5.5</v>
       </c>
@@ -8742,6 +9291,9 @@
       <c r="D342">
         <v>8</v>
       </c>
+      <c r="E342">
+        <v>-0.4</v>
+      </c>
       <c r="F342">
         <v>5.5</v>
       </c>
@@ -8973,6 +9525,9 @@
       <c r="D351">
         <v>17</v>
       </c>
+      <c r="E351">
+        <v>-1.5</v>
+      </c>
       <c r="F351">
         <v>3.9</v>
       </c>
@@ -8996,6 +9551,9 @@
       <c r="D352">
         <v>18</v>
       </c>
+      <c r="E352">
+        <v>-1.4</v>
+      </c>
       <c r="F352">
         <v>4.7</v>
       </c>
@@ -9019,6 +9577,9 @@
       <c r="D353">
         <v>19</v>
       </c>
+      <c r="E353">
+        <v>-0.8</v>
+      </c>
       <c r="F353">
         <v>6.6</v>
       </c>
@@ -9432,6 +9993,9 @@
       <c r="D369">
         <v>4</v>
       </c>
+      <c r="E369">
+        <v>-0.5</v>
+      </c>
       <c r="F369">
         <v>2.8</v>
       </c>
@@ -9455,6 +10019,9 @@
       <c r="D370">
         <v>5</v>
       </c>
+      <c r="E370">
+        <v>-0.1</v>
+      </c>
       <c r="F370">
         <v>3</v>
       </c>
@@ -9764,6 +10331,9 @@
       <c r="D382">
         <v>17</v>
       </c>
+      <c r="E382">
+        <v>-0.2</v>
+      </c>
       <c r="F382">
         <v>4.9</v>
       </c>
@@ -9969,6 +10539,9 @@
       <c r="D390">
         <v>25</v>
       </c>
+      <c r="E390">
+        <v>-0.5</v>
+      </c>
       <c r="F390">
         <v>3.8</v>
       </c>
@@ -10096,6 +10669,9 @@
       <c r="D395">
         <v>30</v>
       </c>
+      <c r="E395">
+        <v>-0.4</v>
+      </c>
       <c r="F395">
         <v>5.3</v>
       </c>
@@ -10119,6 +10695,9 @@
       <c r="D396">
         <v>31</v>
       </c>
+      <c r="E396">
+        <v>-1.6</v>
+      </c>
       <c r="F396">
         <v>5.4</v>
       </c>
@@ -10142,6 +10721,9 @@
       <c r="D397">
         <v>1</v>
       </c>
+      <c r="E397">
+        <v>-0.6</v>
+      </c>
       <c r="F397">
         <v>5.3</v>
       </c>
@@ -10165,6 +10747,9 @@
       <c r="D398">
         <v>2</v>
       </c>
+      <c r="E398">
+        <v>-1</v>
+      </c>
       <c r="F398">
         <v>5.5</v>
       </c>
@@ -10188,6 +10773,9 @@
       <c r="D399">
         <v>3</v>
       </c>
+      <c r="E399">
+        <v>-0.7</v>
+      </c>
       <c r="F399">
         <v>3.6</v>
       </c>
@@ -10211,6 +10799,9 @@
       <c r="D400">
         <v>4</v>
       </c>
+      <c r="E400">
+        <v>-2.3</v>
+      </c>
       <c r="F400">
         <v>3.3</v>
       </c>
@@ -10234,6 +10825,9 @@
       <c r="D401">
         <v>5</v>
       </c>
+      <c r="E401">
+        <v>-2.1</v>
+      </c>
       <c r="F401">
         <v>3.9</v>
       </c>
@@ -10725,6 +11319,9 @@
       <c r="D420">
         <v>24</v>
       </c>
+      <c r="E420">
+        <v>-0.3</v>
+      </c>
       <c r="F420">
         <v>3.6</v>
       </c>
@@ -11268,6 +11865,9 @@
       <c r="D441">
         <v>15</v>
       </c>
+      <c r="E441">
+        <v>-1.3</v>
+      </c>
       <c r="F441">
         <v>1.2</v>
       </c>
@@ -11291,6 +11891,12 @@
       <c r="D442">
         <v>16</v>
       </c>
+      <c r="E442">
+        <v>-0.7</v>
+      </c>
+      <c r="F442">
+        <v>-0.5</v>
+      </c>
       <c r="G442">
         <v>0.9</v>
       </c>
@@ -11340,6 +11946,9 @@
       <c r="E444">
         <v>0.3</v>
       </c>
+      <c r="F444">
+        <v>-2.1</v>
+      </c>
       <c r="G444">
         <v>2.1</v>
       </c>
@@ -11360,6 +11969,12 @@
       <c r="D445">
         <v>19</v>
       </c>
+      <c r="E445">
+        <v>-1.3</v>
+      </c>
+      <c r="F445">
+        <v>-3.3</v>
+      </c>
       <c r="G445">
         <v>3.5</v>
       </c>
@@ -11383,6 +11998,9 @@
       <c r="E446">
         <v>0.7</v>
       </c>
+      <c r="F446">
+        <v>-1.7</v>
+      </c>
       <c r="G446">
         <v>1.8</v>
       </c>
@@ -11403,6 +12021,9 @@
       <c r="D447">
         <v>21</v>
       </c>
+      <c r="E447">
+        <v>-1.1</v>
+      </c>
       <c r="F447">
         <v>0</v>
       </c>
@@ -11426,6 +12047,9 @@
       <c r="D448">
         <v>22</v>
       </c>
+      <c r="E448">
+        <v>-0.9</v>
+      </c>
       <c r="F448">
         <v>2.4</v>
       </c>
@@ -11504,6 +12128,9 @@
       <c r="E451">
         <v>2.9</v>
       </c>
+      <c r="F451">
+        <v>-0.3</v>
+      </c>
       <c r="G451">
         <v>2.9</v>
       </c>
@@ -11524,6 +12151,12 @@
       <c r="D452">
         <v>26</v>
       </c>
+      <c r="E452">
+        <v>-0.1</v>
+      </c>
+      <c r="F452">
+        <v>-2.7</v>
+      </c>
       <c r="G452">
         <v>2.7</v>
       </c>
@@ -11544,6 +12177,12 @@
       <c r="D453">
         <v>27</v>
       </c>
+      <c r="E453">
+        <v>-3</v>
+      </c>
+      <c r="F453">
+        <v>-0.3</v>
+      </c>
       <c r="G453">
         <v>3</v>
       </c>
@@ -11564,6 +12203,9 @@
       <c r="D454">
         <v>28</v>
       </c>
+      <c r="E454">
+        <v>-1.3</v>
+      </c>
       <c r="F454">
         <v>1.2</v>
       </c>
@@ -11639,6 +12281,12 @@
       <c r="D457">
         <v>3</v>
       </c>
+      <c r="E457">
+        <v>-0.5</v>
+      </c>
+      <c r="F457">
+        <v>-1.1</v>
+      </c>
       <c r="G457">
         <v>1.2</v>
       </c>
@@ -11659,6 +12307,9 @@
       <c r="D458">
         <v>4</v>
       </c>
+      <c r="E458">
+        <v>-2.6</v>
+      </c>
       <c r="F458">
         <v>2.3</v>
       </c>
@@ -11682,6 +12333,9 @@
       <c r="D459">
         <v>5</v>
       </c>
+      <c r="E459">
+        <v>-2.7</v>
+      </c>
       <c r="F459">
         <v>3.7</v>
       </c>
@@ -11705,6 +12359,9 @@
       <c r="D460">
         <v>6</v>
       </c>
+      <c r="E460">
+        <v>-2.2</v>
+      </c>
       <c r="F460">
         <v>5.1</v>
       </c>
@@ -11754,6 +12411,12 @@
       <c r="D462">
         <v>8</v>
       </c>
+      <c r="E462">
+        <v>-1.6</v>
+      </c>
+      <c r="F462">
+        <v>-0.1</v>
+      </c>
       <c r="G462">
         <v>1.6</v>
       </c>
@@ -11774,6 +12437,12 @@
       <c r="D463">
         <v>9</v>
       </c>
+      <c r="E463">
+        <v>-1.4</v>
+      </c>
+      <c r="F463">
+        <v>-1.8</v>
+      </c>
       <c r="G463">
         <v>2.3</v>
       </c>
@@ -11794,6 +12463,12 @@
       <c r="D464">
         <v>10</v>
       </c>
+      <c r="E464">
+        <v>-0.6</v>
+      </c>
+      <c r="F464">
+        <v>-1.5</v>
+      </c>
       <c r="G464">
         <v>1.6</v>
       </c>
@@ -11814,6 +12489,12 @@
       <c r="D465">
         <v>11</v>
       </c>
+      <c r="E465">
+        <v>-2.4</v>
+      </c>
+      <c r="F465">
+        <v>-1.9</v>
+      </c>
       <c r="G465">
         <v>3</v>
       </c>
@@ -11834,6 +12515,12 @@
       <c r="D466">
         <v>12</v>
       </c>
+      <c r="E466">
+        <v>-4.6</v>
+      </c>
+      <c r="F466">
+        <v>-3.9</v>
+      </c>
       <c r="G466">
         <v>6.1</v>
       </c>
@@ -11854,6 +12541,12 @@
       <c r="D467">
         <v>13</v>
       </c>
+      <c r="E467">
+        <v>-3.4</v>
+      </c>
+      <c r="F467">
+        <v>-2.1</v>
+      </c>
       <c r="G467">
         <v>4</v>
       </c>
@@ -11874,6 +12567,12 @@
       <c r="D468">
         <v>14</v>
       </c>
+      <c r="E468">
+        <v>-3.5</v>
+      </c>
+      <c r="F468">
+        <v>-0.7</v>
+      </c>
       <c r="G468">
         <v>3.5</v>
       </c>
@@ -11894,6 +12593,9 @@
       <c r="D469">
         <v>15</v>
       </c>
+      <c r="E469">
+        <v>-1.1</v>
+      </c>
       <c r="F469">
         <v>0.8</v>
       </c>
@@ -11917,6 +12619,12 @@
       <c r="D470">
         <v>16</v>
       </c>
+      <c r="E470">
+        <v>-1.9</v>
+      </c>
+      <c r="F470">
+        <v>-1.1</v>
+      </c>
       <c r="G470">
         <v>2.2</v>
       </c>
@@ -11937,6 +12645,12 @@
       <c r="D471">
         <v>17</v>
       </c>
+      <c r="E471">
+        <v>-3.1</v>
+      </c>
+      <c r="F471">
+        <v>-1.3</v>
+      </c>
       <c r="G471">
         <v>3.3</v>
       </c>
@@ -11957,6 +12671,9 @@
       <c r="D472">
         <v>18</v>
       </c>
+      <c r="E472">
+        <v>-4.1</v>
+      </c>
       <c r="F472">
         <v>0.5</v>
       </c>
@@ -11980,6 +12697,9 @@
       <c r="D473">
         <v>19</v>
       </c>
+      <c r="E473">
+        <v>-1.6</v>
+      </c>
       <c r="F473">
         <v>1.8</v>
       </c>
@@ -12055,6 +12775,12 @@
       <c r="D476">
         <v>22</v>
       </c>
+      <c r="E476">
+        <v>-1.5</v>
+      </c>
+      <c r="F476">
+        <v>-0.1</v>
+      </c>
       <c r="G476">
         <v>1.5</v>
       </c>
@@ -12075,6 +12801,12 @@
       <c r="D477">
         <v>23</v>
       </c>
+      <c r="E477">
+        <v>-4.8</v>
+      </c>
+      <c r="F477">
+        <v>-2.2</v>
+      </c>
       <c r="G477">
         <v>5.3</v>
       </c>
@@ -12095,6 +12827,9 @@
       <c r="D478">
         <v>24</v>
       </c>
+      <c r="E478">
+        <v>-1.5</v>
+      </c>
       <c r="F478">
         <v>1.1</v>
       </c>
@@ -12121,6 +12856,9 @@
       <c r="E479">
         <v>2.5</v>
       </c>
+      <c r="F479">
+        <v>-0.4</v>
+      </c>
       <c r="G479">
         <v>2.5</v>
       </c>
@@ -12219,6 +12957,9 @@
       <c r="D483">
         <v>29</v>
       </c>
+      <c r="E483">
+        <v>-1.7</v>
+      </c>
       <c r="F483">
         <v>2</v>
       </c>
@@ -12323,6 +13064,9 @@
       <c r="E487">
         <v>0.9</v>
       </c>
+      <c r="F487">
+        <v>-0.4</v>
+      </c>
       <c r="G487">
         <v>1</v>
       </c>
@@ -12343,6 +13087,12 @@
       <c r="D488">
         <v>3</v>
       </c>
+      <c r="E488">
+        <v>-0.2</v>
+      </c>
+      <c r="F488">
+        <v>-1.3</v>
+      </c>
       <c r="G488">
         <v>1.3</v>
       </c>
@@ -12363,6 +13113,12 @@
       <c r="D489">
         <v>4</v>
       </c>
+      <c r="E489">
+        <v>-0.2</v>
+      </c>
+      <c r="F489">
+        <v>-1.4</v>
+      </c>
       <c r="G489">
         <v>1.4</v>
       </c>
@@ -12386,6 +13142,9 @@
       <c r="E490">
         <v>0.1</v>
       </c>
+      <c r="F490">
+        <v>-2</v>
+      </c>
       <c r="G490">
         <v>2</v>
       </c>
@@ -12406,6 +13165,9 @@
       <c r="D491">
         <v>6</v>
       </c>
+      <c r="E491">
+        <v>-0.2</v>
+      </c>
       <c r="F491">
         <v>0.2</v>
       </c>
@@ -12429,6 +13191,12 @@
       <c r="D492">
         <v>7</v>
       </c>
+      <c r="E492">
+        <v>-0.9</v>
+      </c>
+      <c r="F492">
+        <v>-2.9</v>
+      </c>
       <c r="G492">
         <v>3</v>
       </c>
@@ -12449,6 +13217,12 @@
       <c r="D493">
         <v>8</v>
       </c>
+      <c r="E493">
+        <v>-1.8</v>
+      </c>
+      <c r="F493">
+        <v>-3.6</v>
+      </c>
       <c r="G493">
         <v>4</v>
       </c>
@@ -12472,6 +13246,9 @@
       <c r="E494">
         <v>0.5</v>
       </c>
+      <c r="F494">
+        <v>-1.6</v>
+      </c>
       <c r="G494">
         <v>1.7</v>
       </c>
@@ -12495,6 +13272,9 @@
       <c r="E495">
         <v>0.9</v>
       </c>
+      <c r="F495">
+        <v>-5.2</v>
+      </c>
       <c r="G495">
         <v>5.3</v>
       </c>
@@ -12515,6 +13295,12 @@
       <c r="D496">
         <v>11</v>
       </c>
+      <c r="E496">
+        <v>-0.6</v>
+      </c>
+      <c r="F496">
+        <v>-4.7</v>
+      </c>
       <c r="G496">
         <v>4.7</v>
       </c>
@@ -12535,6 +13321,12 @@
       <c r="D497">
         <v>12</v>
       </c>
+      <c r="E497">
+        <v>-0.4</v>
+      </c>
+      <c r="F497">
+        <v>-5.5</v>
+      </c>
       <c r="G497">
         <v>5.5</v>
       </c>
@@ -12558,6 +13350,9 @@
       <c r="E498">
         <v>0.1</v>
       </c>
+      <c r="F498">
+        <v>-4.1</v>
+      </c>
       <c r="G498">
         <v>4.1</v>
       </c>
@@ -12578,6 +13373,12 @@
       <c r="D499">
         <v>14</v>
       </c>
+      <c r="E499">
+        <v>-0.1</v>
+      </c>
+      <c r="F499">
+        <v>-1.4</v>
+      </c>
       <c r="G499">
         <v>1.4</v>
       </c>
@@ -12598,6 +13399,12 @@
       <c r="D500">
         <v>15</v>
       </c>
+      <c r="E500">
+        <v>-0.3</v>
+      </c>
+      <c r="F500">
+        <v>-0.9</v>
+      </c>
       <c r="G500">
         <v>0.9</v>
       </c>
@@ -12618,6 +13425,12 @@
       <c r="D501">
         <v>16</v>
       </c>
+      <c r="E501">
+        <v>-0.8</v>
+      </c>
+      <c r="F501">
+        <v>-1.4</v>
+      </c>
       <c r="G501">
         <v>1.6</v>
       </c>
@@ -12638,6 +13451,12 @@
       <c r="D502">
         <v>17</v>
       </c>
+      <c r="E502">
+        <v>-0.7</v>
+      </c>
+      <c r="F502">
+        <v>-2.8</v>
+      </c>
       <c r="G502">
         <v>2.9</v>
       </c>
@@ -12658,6 +13477,12 @@
       <c r="D503">
         <v>18</v>
       </c>
+      <c r="E503">
+        <v>-2.9</v>
+      </c>
+      <c r="F503">
+        <v>-2.8</v>
+      </c>
       <c r="G503">
         <v>4</v>
       </c>
@@ -12678,6 +13503,12 @@
       <c r="D504">
         <v>19</v>
       </c>
+      <c r="E504">
+        <v>-5.8</v>
+      </c>
+      <c r="F504">
+        <v>-3.3</v>
+      </c>
       <c r="G504">
         <v>6.7</v>
       </c>
@@ -12698,6 +13529,12 @@
       <c r="D505">
         <v>20</v>
       </c>
+      <c r="E505">
+        <v>-4.4</v>
+      </c>
+      <c r="F505">
+        <v>-3.8</v>
+      </c>
       <c r="G505">
         <v>5.8</v>
       </c>
@@ -12718,6 +13555,12 @@
       <c r="D506">
         <v>21</v>
       </c>
+      <c r="E506">
+        <v>-5.6</v>
+      </c>
+      <c r="F506">
+        <v>-2.9</v>
+      </c>
       <c r="G506">
         <v>6.3</v>
       </c>
@@ -12738,6 +13581,12 @@
       <c r="D507">
         <v>22</v>
       </c>
+      <c r="E507">
+        <v>-5.9</v>
+      </c>
+      <c r="F507">
+        <v>-2.8</v>
+      </c>
       <c r="G507">
         <v>6.6</v>
       </c>
@@ -12758,6 +13607,12 @@
       <c r="D508">
         <v>23</v>
       </c>
+      <c r="E508">
+        <v>-2.9</v>
+      </c>
+      <c r="F508">
+        <v>-2</v>
+      </c>
       <c r="G508">
         <v>3.6</v>
       </c>
@@ -12778,6 +13633,12 @@
       <c r="D509">
         <v>24</v>
       </c>
+      <c r="E509">
+        <v>-5.9</v>
+      </c>
+      <c r="F509">
+        <v>-4</v>
+      </c>
       <c r="G509">
         <v>7.1</v>
       </c>
@@ -12902,6 +13763,9 @@
       <c r="D514">
         <v>14</v>
       </c>
+      <c r="E514">
+        <v>-0.8</v>
+      </c>
       <c r="F514">
         <v>1.8</v>
       </c>
@@ -13393,6 +14257,9 @@
       <c r="D533">
         <v>2</v>
       </c>
+      <c r="E533">
+        <v>-1.2</v>
+      </c>
       <c r="F533">
         <v>0</v>
       </c>
@@ -13416,6 +14283,9 @@
       <c r="D534">
         <v>3</v>
       </c>
+      <c r="E534">
+        <v>-2.1</v>
+      </c>
       <c r="F534">
         <v>1.2</v>
       </c>
@@ -13439,6 +14309,9 @@
       <c r="D535">
         <v>4</v>
       </c>
+      <c r="E535">
+        <v>-2.6</v>
+      </c>
       <c r="F535">
         <v>1.3</v>
       </c>
@@ -13465,6 +14338,9 @@
       <c r="E536">
         <v>0.4</v>
       </c>
+      <c r="F536">
+        <v>-2.1</v>
+      </c>
       <c r="G536">
         <v>2.1</v>
       </c>
@@ -13488,6 +14364,9 @@
       <c r="E537">
         <v>1.8</v>
       </c>
+      <c r="F537">
+        <v>-0.9</v>
+      </c>
       <c r="G537">
         <v>2</v>
       </c>
@@ -13563,6 +14442,9 @@
       <c r="E540">
         <v>3.8</v>
       </c>
+      <c r="F540">
+        <v>-0.5</v>
+      </c>
       <c r="G540">
         <v>3.9</v>
       </c>
@@ -13638,6 +14520,9 @@
       <c r="E543">
         <v>3.3</v>
       </c>
+      <c r="F543">
+        <v>-0.2</v>
+      </c>
       <c r="G543">
         <v>3.3</v>
       </c>
@@ -13661,6 +14546,9 @@
       <c r="E544">
         <v>3</v>
       </c>
+      <c r="F544">
+        <v>-0.3</v>
+      </c>
       <c r="G544">
         <v>3</v>
       </c>
@@ -13889,6 +14777,9 @@
       <c r="D553">
         <v>22</v>
       </c>
+      <c r="E553">
+        <v>-0.1</v>
+      </c>
       <c r="F553">
         <v>6.3</v>
       </c>
@@ -15836,6 +16727,9 @@
       <c r="D628">
         <v>5</v>
       </c>
+      <c r="E628">
+        <v>-0.7</v>
+      </c>
       <c r="F628">
         <v>1.1</v>
       </c>
@@ -15859,6 +16753,9 @@
       <c r="D629">
         <v>6</v>
       </c>
+      <c r="E629">
+        <v>-1.9</v>
+      </c>
       <c r="F629">
         <v>3.9</v>
       </c>
@@ -15960,6 +16857,9 @@
       <c r="D633">
         <v>10</v>
       </c>
+      <c r="E633">
+        <v>-1.4</v>
+      </c>
       <c r="F633">
         <v>5.9</v>
       </c>
@@ -15983,6 +16883,9 @@
       <c r="D634">
         <v>11</v>
       </c>
+      <c r="E634">
+        <v>-0.6</v>
+      </c>
       <c r="F634">
         <v>5.4</v>
       </c>
@@ -16188,6 +17091,9 @@
       <c r="D642">
         <v>19</v>
       </c>
+      <c r="E642">
+        <v>-0.2</v>
+      </c>
       <c r="F642">
         <v>3.6</v>
       </c>
@@ -16211,6 +17117,9 @@
       <c r="D643">
         <v>20</v>
       </c>
+      <c r="E643">
+        <v>-0.4</v>
+      </c>
       <c r="F643">
         <v>2.3</v>
       </c>
@@ -16442,6 +17351,9 @@
       <c r="D652">
         <v>29</v>
       </c>
+      <c r="E652">
+        <v>-0.4</v>
+      </c>
       <c r="F652">
         <v>3.9</v>
       </c>
@@ -16465,6 +17377,12 @@
       <c r="D653">
         <v>30</v>
       </c>
+      <c r="E653">
+        <v>-0.1</v>
+      </c>
+      <c r="F653">
+        <v>-1.1</v>
+      </c>
       <c r="G653">
         <v>1.1</v>
       </c>
@@ -16485,6 +17403,12 @@
       <c r="D654">
         <v>1</v>
       </c>
+      <c r="E654">
+        <v>-2.1</v>
+      </c>
+      <c r="F654">
+        <v>-0.2</v>
+      </c>
       <c r="G654">
         <v>2.1</v>
       </c>
@@ -16505,6 +17429,9 @@
       <c r="D655">
         <v>2</v>
       </c>
+      <c r="E655">
+        <v>-1.9</v>
+      </c>
       <c r="F655">
         <v>0.8</v>
       </c>
@@ -16528,6 +17455,9 @@
       <c r="D656">
         <v>3</v>
       </c>
+      <c r="E656">
+        <v>-0.1</v>
+      </c>
       <c r="F656">
         <v>1.9</v>
       </c>
@@ -16629,6 +17559,9 @@
       <c r="D660">
         <v>7</v>
       </c>
+      <c r="E660">
+        <v>-0.9</v>
+      </c>
       <c r="F660">
         <v>2.1</v>
       </c>
@@ -16652,6 +17585,9 @@
       <c r="D661">
         <v>8</v>
       </c>
+      <c r="E661">
+        <v>-0.1</v>
+      </c>
       <c r="F661">
         <v>3.8</v>
       </c>
@@ -16675,6 +17611,9 @@
       <c r="D662">
         <v>9</v>
       </c>
+      <c r="E662">
+        <v>-0.3</v>
+      </c>
       <c r="F662">
         <v>2.2</v>
       </c>
@@ -16698,6 +17637,9 @@
       <c r="D663">
         <v>10</v>
       </c>
+      <c r="E663">
+        <v>-0.5</v>
+      </c>
       <c r="F663">
         <v>2</v>
       </c>
@@ -16721,6 +17663,9 @@
       <c r="D664">
         <v>11</v>
       </c>
+      <c r="E664">
+        <v>-0.2</v>
+      </c>
       <c r="F664">
         <v>1.5</v>
       </c>
@@ -16744,6 +17689,9 @@
       <c r="D665">
         <v>12</v>
       </c>
+      <c r="E665">
+        <v>-0.2</v>
+      </c>
       <c r="F665">
         <v>0.9</v>
       </c>
@@ -16767,6 +17715,9 @@
       <c r="D666">
         <v>13</v>
       </c>
+      <c r="E666">
+        <v>-0.3</v>
+      </c>
       <c r="F666">
         <v>0.5</v>
       </c>
@@ -16793,6 +17744,9 @@
       <c r="E667">
         <v>0.1</v>
       </c>
+      <c r="F667">
+        <v>-1.5</v>
+      </c>
       <c r="G667">
         <v>1.5</v>
       </c>
@@ -16813,6 +17767,12 @@
       <c r="D668">
         <v>15</v>
       </c>
+      <c r="E668">
+        <v>-0.3</v>
+      </c>
+      <c r="F668">
+        <v>-1.4</v>
+      </c>
       <c r="G668">
         <v>1.5</v>
       </c>
@@ -16859,6 +17819,9 @@
       <c r="D670">
         <v>17</v>
       </c>
+      <c r="E670">
+        <v>-0.7</v>
+      </c>
       <c r="F670">
         <v>0.9</v>
       </c>
@@ -16882,6 +17845,9 @@
       <c r="D671">
         <v>18</v>
       </c>
+      <c r="E671">
+        <v>-0.7</v>
+      </c>
       <c r="F671">
         <v>1.1</v>
       </c>
@@ -17139,6 +18105,9 @@
       <c r="D681">
         <v>28</v>
       </c>
+      <c r="E681">
+        <v>-0.9</v>
+      </c>
       <c r="F681">
         <v>4.5</v>
       </c>
@@ -17162,6 +18131,9 @@
       <c r="D682">
         <v>29</v>
       </c>
+      <c r="E682">
+        <v>-2.4</v>
+      </c>
       <c r="F682">
         <v>3.7</v>
       </c>
@@ -17185,6 +18157,12 @@
       <c r="D683">
         <v>30</v>
       </c>
+      <c r="E683">
+        <v>-2.3</v>
+      </c>
+      <c r="F683">
+        <v>-0.7</v>
+      </c>
       <c r="G683">
         <v>2.4</v>
       </c>
@@ -17205,6 +18183,12 @@
       <c r="D684">
         <v>31</v>
       </c>
+      <c r="E684">
+        <v>-1.3</v>
+      </c>
+      <c r="F684">
+        <v>-0.2</v>
+      </c>
       <c r="G684">
         <v>1.4</v>
       </c>
@@ -17381,6 +18365,9 @@
       <c r="D691">
         <v>7</v>
       </c>
+      <c r="E691">
+        <v>-0.1</v>
+      </c>
       <c r="F691">
         <v>3.8</v>
       </c>
@@ -17404,6 +18391,9 @@
       <c r="D692">
         <v>8</v>
       </c>
+      <c r="E692">
+        <v>-2.4</v>
+      </c>
       <c r="F692">
         <v>0.9</v>
       </c>
@@ -17430,6 +18420,9 @@
       <c r="E693">
         <v>2.4</v>
       </c>
+      <c r="F693">
+        <v>-1.8</v>
+      </c>
       <c r="G693">
         <v>3.1</v>
       </c>
@@ -17453,6 +18446,9 @@
       <c r="E694">
         <v>3</v>
       </c>
+      <c r="F694">
+        <v>-2.7</v>
+      </c>
       <c r="G694">
         <v>4</v>
       </c>
@@ -17476,6 +18472,9 @@
       <c r="E695">
         <v>7</v>
       </c>
+      <c r="F695">
+        <v>-0.5</v>
+      </c>
       <c r="G695">
         <v>7</v>
       </c>
@@ -17499,6 +18498,9 @@
       <c r="E696">
         <v>2.6</v>
       </c>
+      <c r="F696">
+        <v>-3.2</v>
+      </c>
       <c r="G696">
         <v>4.2</v>
       </c>
@@ -17600,6 +18602,9 @@
       <c r="E700">
         <v>0.7</v>
       </c>
+      <c r="F700">
+        <v>-0.3</v>
+      </c>
       <c r="G700">
         <v>0.8</v>
       </c>
@@ -17620,6 +18625,12 @@
       <c r="D701">
         <v>17</v>
       </c>
+      <c r="E701">
+        <v>-0.6</v>
+      </c>
+      <c r="F701">
+        <v>-2.1</v>
+      </c>
       <c r="G701">
         <v>2.2</v>
       </c>
@@ -17640,6 +18651,12 @@
       <c r="D702">
         <v>18</v>
       </c>
+      <c r="E702">
+        <v>-2.4</v>
+      </c>
+      <c r="F702">
+        <v>-1.4</v>
+      </c>
       <c r="G702">
         <v>2.8</v>
       </c>
@@ -17660,6 +18677,9 @@
       <c r="D703">
         <v>19</v>
       </c>
+      <c r="E703">
+        <v>-0.9</v>
+      </c>
       <c r="F703">
         <v>1.7</v>
       </c>
@@ -17735,6 +18755,12 @@
       <c r="D706">
         <v>22</v>
       </c>
+      <c r="E706">
+        <v>-1.3</v>
+      </c>
+      <c r="F706">
+        <v>-4.3</v>
+      </c>
       <c r="G706">
         <v>4.5</v>
       </c>
@@ -17755,6 +18781,12 @@
       <c r="D707">
         <v>23</v>
       </c>
+      <c r="E707">
+        <v>-2.9</v>
+      </c>
+      <c r="F707">
+        <v>-3.3</v>
+      </c>
       <c r="G707">
         <v>4.4</v>
       </c>
@@ -17775,6 +18807,12 @@
       <c r="D708">
         <v>24</v>
       </c>
+      <c r="E708">
+        <v>-1.6</v>
+      </c>
+      <c r="F708">
+        <v>-2.9</v>
+      </c>
       <c r="G708">
         <v>3.3</v>
       </c>
@@ -17795,6 +18833,12 @@
       <c r="D709">
         <v>25</v>
       </c>
+      <c r="E709">
+        <v>-0.8</v>
+      </c>
+      <c r="F709">
+        <v>-2.2</v>
+      </c>
       <c r="G709">
         <v>2.3</v>
       </c>
@@ -17815,6 +18859,12 @@
       <c r="D710">
         <v>9</v>
       </c>
+      <c r="E710">
+        <v>-0.3</v>
+      </c>
+      <c r="F710">
+        <v>-2.8</v>
+      </c>
       <c r="G710">
         <v>2.8</v>
       </c>
@@ -17835,6 +18885,12 @@
       <c r="D711">
         <v>10</v>
       </c>
+      <c r="E711">
+        <v>-2.1</v>
+      </c>
+      <c r="F711">
+        <v>-0.2</v>
+      </c>
       <c r="G711">
         <v>2.2</v>
       </c>
@@ -17855,6 +18911,9 @@
       <c r="D712">
         <v>11</v>
       </c>
+      <c r="E712">
+        <v>-4.5</v>
+      </c>
       <c r="F712">
         <v>1.1</v>
       </c>
@@ -17878,6 +18937,9 @@
       <c r="D713">
         <v>12</v>
       </c>
+      <c r="E713">
+        <v>-2.2</v>
+      </c>
       <c r="F713">
         <v>2.1</v>
       </c>
@@ -17901,6 +18963,9 @@
       <c r="D714">
         <v>13</v>
       </c>
+      <c r="E714">
+        <v>-1.8</v>
+      </c>
       <c r="F714">
         <v>0.8</v>
       </c>
@@ -17927,6 +18992,9 @@
       <c r="E715">
         <v>0.8</v>
       </c>
+      <c r="F715">
+        <v>-1.1</v>
+      </c>
       <c r="G715">
         <v>1.4</v>
       </c>
@@ -17947,6 +19015,12 @@
       <c r="D716">
         <v>15</v>
       </c>
+      <c r="E716">
+        <v>-0.1</v>
+      </c>
+      <c r="F716">
+        <v>-3.4</v>
+      </c>
       <c r="G716">
         <v>3.4</v>
       </c>
@@ -17967,6 +19041,12 @@
       <c r="D717">
         <v>16</v>
       </c>
+      <c r="E717">
+        <v>-1.5</v>
+      </c>
+      <c r="F717">
+        <v>-3.8</v>
+      </c>
       <c r="G717">
         <v>4.1</v>
       </c>
@@ -17987,6 +19067,12 @@
       <c r="D718">
         <v>17</v>
       </c>
+      <c r="E718">
+        <v>-3.8</v>
+      </c>
+      <c r="F718">
+        <v>-1.8</v>
+      </c>
       <c r="G718">
         <v>4.2</v>
       </c>
@@ -18007,6 +19093,12 @@
       <c r="D719">
         <v>18</v>
       </c>
+      <c r="E719">
+        <v>-4.2</v>
+      </c>
+      <c r="F719">
+        <v>-1.8</v>
+      </c>
       <c r="G719">
         <v>4.6</v>
       </c>
@@ -18027,6 +19119,12 @@
       <c r="D720">
         <v>19</v>
       </c>
+      <c r="E720">
+        <v>-1.9</v>
+      </c>
+      <c r="F720">
+        <v>-3.8</v>
+      </c>
       <c r="G720">
         <v>4.2</v>
       </c>
@@ -18047,6 +19145,12 @@
       <c r="D721">
         <v>20</v>
       </c>
+      <c r="E721">
+        <v>-1.2</v>
+      </c>
+      <c r="F721">
+        <v>-3.5</v>
+      </c>
       <c r="G721">
         <v>3.7</v>
       </c>
@@ -18067,6 +19171,12 @@
       <c r="D722">
         <v>21</v>
       </c>
+      <c r="E722">
+        <v>-1.2</v>
+      </c>
+      <c r="F722">
+        <v>-1.1</v>
+      </c>
       <c r="G722">
         <v>1.6</v>
       </c>
@@ -18087,6 +19197,12 @@
       <c r="D723">
         <v>22</v>
       </c>
+      <c r="E723">
+        <v>-2</v>
+      </c>
+      <c r="F723">
+        <v>-0.8</v>
+      </c>
       <c r="G723">
         <v>2.1</v>
       </c>
@@ -18107,6 +19223,12 @@
       <c r="D724">
         <v>23</v>
       </c>
+      <c r="E724">
+        <v>-0.2</v>
+      </c>
+      <c r="F724">
+        <v>-1.6</v>
+      </c>
       <c r="G724">
         <v>1.7</v>
       </c>
@@ -18127,6 +19249,12 @@
       <c r="D725">
         <v>24</v>
       </c>
+      <c r="E725">
+        <v>-0.9</v>
+      </c>
+      <c r="F725">
+        <v>-2.7</v>
+      </c>
       <c r="G725">
         <v>2.8</v>
       </c>
@@ -18147,6 +19275,12 @@
       <c r="D726">
         <v>25</v>
       </c>
+      <c r="E726">
+        <v>-2.7</v>
+      </c>
+      <c r="F726">
+        <v>-1.6</v>
+      </c>
       <c r="G726">
         <v>3.2</v>
       </c>
@@ -18167,6 +19301,9 @@
       <c r="D727">
         <v>26</v>
       </c>
+      <c r="E727">
+        <v>-3.5</v>
+      </c>
       <c r="F727">
         <v>0</v>
       </c>
@@ -18190,6 +19327,9 @@
       <c r="D728">
         <v>27</v>
       </c>
+      <c r="E728">
+        <v>-2.1</v>
+      </c>
       <c r="F728">
         <v>1.7</v>
       </c>
@@ -18213,6 +19353,9 @@
       <c r="D729">
         <v>28</v>
       </c>
+      <c r="E729">
+        <v>-2.4</v>
+      </c>
       <c r="F729">
         <v>0.5</v>
       </c>
@@ -18236,6 +19379,12 @@
       <c r="D730">
         <v>29</v>
       </c>
+      <c r="E730">
+        <v>-2.8</v>
+      </c>
+      <c r="F730">
+        <v>-0.4</v>
+      </c>
       <c r="G730">
         <v>2.8</v>
       </c>
@@ -18256,6 +19405,12 @@
       <c r="D731">
         <v>30</v>
       </c>
+      <c r="E731">
+        <v>-1.2</v>
+      </c>
+      <c r="F731">
+        <v>-1.2</v>
+      </c>
       <c r="G731">
         <v>1.7</v>
       </c>
@@ -18276,6 +19431,12 @@
       <c r="D732">
         <v>31</v>
       </c>
+      <c r="E732">
+        <v>-0.7</v>
+      </c>
+      <c r="F732">
+        <v>-1</v>
+      </c>
       <c r="G732">
         <v>1.2</v>
       </c>
@@ -18296,6 +19457,12 @@
       <c r="D733">
         <v>1</v>
       </c>
+      <c r="E733">
+        <v>-1.6</v>
+      </c>
+      <c r="F733">
+        <v>-1.3</v>
+      </c>
       <c r="G733">
         <v>2</v>
       </c>
@@ -18316,6 +19483,12 @@
       <c r="D734">
         <v>2</v>
       </c>
+      <c r="E734">
+        <v>-2.9</v>
+      </c>
+      <c r="F734">
+        <v>-1.1</v>
+      </c>
       <c r="G734">
         <v>3</v>
       </c>
@@ -18336,6 +19509,12 @@
       <c r="D735">
         <v>3</v>
       </c>
+      <c r="E735">
+        <v>-2.5</v>
+      </c>
+      <c r="F735">
+        <v>-0.3</v>
+      </c>
       <c r="G735">
         <v>2.5</v>
       </c>
@@ -18356,6 +19535,12 @@
       <c r="D736">
         <v>4</v>
       </c>
+      <c r="E736">
+        <v>-0.1</v>
+      </c>
+      <c r="F736">
+        <v>-1.1</v>
+      </c>
       <c r="G736">
         <v>1.1</v>
       </c>
@@ -18379,6 +19564,9 @@
       <c r="E737">
         <v>1.4</v>
       </c>
+      <c r="F737">
+        <v>-1.8</v>
+      </c>
       <c r="G737">
         <v>2.2</v>
       </c>
@@ -18402,6 +19590,9 @@
       <c r="E738">
         <v>0.7</v>
       </c>
+      <c r="F738">
+        <v>-4.2</v>
+      </c>
       <c r="G738">
         <v>4.2</v>
       </c>
@@ -18425,6 +19616,9 @@
       <c r="E739">
         <v>2.8</v>
       </c>
+      <c r="F739">
+        <v>-3.8</v>
+      </c>
       <c r="G739">
         <v>4.7</v>
       </c>
@@ -18445,6 +19639,12 @@
       <c r="D740">
         <v>6</v>
       </c>
+      <c r="E740">
+        <v>-2.4</v>
+      </c>
+      <c r="F740">
+        <v>-0.3</v>
+      </c>
       <c r="G740">
         <v>2.5</v>
       </c>
@@ -18465,6 +19665,12 @@
       <c r="D741">
         <v>7</v>
       </c>
+      <c r="E741">
+        <v>-3</v>
+      </c>
+      <c r="F741">
+        <v>-0.8</v>
+      </c>
       <c r="G741">
         <v>3.1</v>
       </c>
@@ -18485,6 +19691,12 @@
       <c r="D742">
         <v>8</v>
       </c>
+      <c r="E742">
+        <v>-2.8</v>
+      </c>
+      <c r="F742">
+        <v>-1</v>
+      </c>
       <c r="G742">
         <v>2.9</v>
       </c>
@@ -18505,6 +19717,9 @@
       <c r="D743">
         <v>9</v>
       </c>
+      <c r="E743">
+        <v>-3</v>
+      </c>
       <c r="F743">
         <v>1</v>
       </c>
@@ -18583,6 +19798,9 @@
       <c r="E746">
         <v>1.6</v>
       </c>
+      <c r="F746">
+        <v>-2.5</v>
+      </c>
       <c r="G746">
         <v>3</v>
       </c>
@@ -18603,6 +19821,12 @@
       <c r="D747">
         <v>13</v>
       </c>
+      <c r="E747">
+        <v>-0.7</v>
+      </c>
+      <c r="F747">
+        <v>-4.4</v>
+      </c>
       <c r="G747">
         <v>4.4</v>
       </c>
@@ -18623,6 +19847,12 @@
       <c r="D748">
         <v>14</v>
       </c>
+      <c r="E748">
+        <v>-1.9</v>
+      </c>
+      <c r="F748">
+        <v>-3.8</v>
+      </c>
       <c r="G748">
         <v>4.3</v>
       </c>
@@ -18643,6 +19873,12 @@
       <c r="D749">
         <v>15</v>
       </c>
+      <c r="E749">
+        <v>-1.1</v>
+      </c>
+      <c r="F749">
+        <v>-3.8</v>
+      </c>
       <c r="G749">
         <v>4</v>
       </c>
@@ -18666,6 +19902,9 @@
       <c r="E750">
         <v>1</v>
       </c>
+      <c r="F750">
+        <v>-3.2</v>
+      </c>
       <c r="G750">
         <v>3.3</v>
       </c>
@@ -18686,6 +19925,12 @@
       <c r="D751">
         <v>17</v>
       </c>
+      <c r="E751">
+        <v>-0.1</v>
+      </c>
+      <c r="F751">
+        <v>-2.5</v>
+      </c>
       <c r="G751">
         <v>2.5</v>
       </c>
@@ -18706,6 +19951,12 @@
       <c r="D752">
         <v>18</v>
       </c>
+      <c r="E752">
+        <v>-0.9</v>
+      </c>
+      <c r="F752">
+        <v>-1.5</v>
+      </c>
       <c r="G752">
         <v>1.7</v>
       </c>
@@ -18729,6 +19980,9 @@
       <c r="E753">
         <v>0.1</v>
       </c>
+      <c r="F753">
+        <v>-2.5</v>
+      </c>
       <c r="G753">
         <v>2.5</v>
       </c>
@@ -18752,6 +20006,9 @@
       <c r="E754">
         <v>2.3</v>
       </c>
+      <c r="F754">
+        <v>-0.4</v>
+      </c>
       <c r="G754">
         <v>2.3</v>
       </c>
@@ -18775,6 +20032,9 @@
       <c r="E755">
         <v>2.4</v>
       </c>
+      <c r="F755">
+        <v>-3.5</v>
+      </c>
       <c r="G755">
         <v>4.2</v>
       </c>
@@ -18794,6 +20054,12 @@
       </c>
       <c r="D756">
         <v>22</v>
+      </c>
+      <c r="E756">
+        <v>-0.3</v>
+      </c>
+      <c r="F756">
+        <v>-4.4</v>
       </c>
       <c r="G756">
         <v>4.4</v>

</xml_diff>